<commit_message>
M03: fix HTML/PPTX prompt mismatch, switch to drag-and-drop xlsx workflow, make Latihan header prominent site-wide
</commit_message>
<xml_diff>
--- a/Content-Marketing/M03-Konten-Instagram/cm-kalender-konten.xlsx
+++ b/Content-Marketing/M03-Konten-Instagram/cm-kalender-konten.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="45">
   <si>
     <t xml:space="preserve">Kalender Konten Instagram — Kreasi Konten Pemasaran (Belajar Claude)</t>
   </si>
@@ -131,19 +131,13 @@
     <t xml:space="preserve">2. Buka Claude Project kamu (yang sudah tahu positioning dari Modul 1 &amp; katalog produk dari Modul 2).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Copy kolom No sampai Jam Post (A:F) dari baris 10 sampai 24 -- 6 kolom ini kerangka kalendermu, bukan yang mau digenerate Claude.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Jalankan prompt ini di Claude (paste kolom yang kamu copy di bagian yang ditandai):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   "Ini kerangka kalender bulan [bulan] saya (No | Minggu | Hari | Tanggal | Jam Post | Kategori):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [paste kolom A-F dari baris 10-24 di sini]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Untuk tiap baris, sesuai Kategori yang sudah ada, buatkan: (1) ide Tema yang spesifik dan menarik -- jangan generic, (2) Format post yang paling cocok untuk ide itu (Foto Produk/Carousel/Reels/Story/Quote), (3) Caption maks 80 kata (Hook-Value/Cerita-CTA), (4) 8 Hashtag. Cocokkan lewat kolom No, jangan ubah urutan. Output tabel: No | Tema | Format | Caption | Hashtag."</t>
+    <t xml:space="preserve">3. Lampirkan file cm-kalender-konten.xlsx ini langsung ke chat Claude (drag &amp; drop) -- tidak perlu copy-paste kolom manual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Jalankan prompt ini di Claude:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   "Ini file kalender kontenku, tab Kalender Konten. Untuk baris 10 sampai 24, sesuai Kategori yang sudah ada di tiap baris, buatkan: (1) ide Tema yang spesifik dan menarik -- jangan generic, (2) Format post yang paling cocok untuk ide itu (Foto Produk/Carousel/Reels/Story/Quote), (3) Caption maks 80 kata (Hook-Value/Cerita-CTA), (4) 8 Hashtag. Cocokkan lewat kolom No, jangan ubah urutan. Output tabel: No | Tema | Format | Caption | Hashtag."</t>
   </si>
   <si>
     <t xml:space="preserve">5. Paste hasil Claude ke kolom Tema, Format, Caption, dan Hashtag (kolom G-J) sesuai nomor barisnya -- jangan asal urut, cocokkan No-nya.</t>
@@ -364,16 +358,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -385,7 +383,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -750,702 +748,702 @@
   <dimension ref="A1:K24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <f aca="false">COUNTA($F$9:$F$24)</f>
         <v>16</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <f aca="false">COUNTIF($F$9:$F$24,"Produk")</f>
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF($F$9:$F$24,"Edukasi")</f>
         <v>5</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <f aca="false">COUNTIF($F$9:$F$24,"BTS")</f>
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <f aca="false">COUNTIF($F$9:$F$24,"Testimoni")</f>
         <v>2</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <f aca="false">COUNTIF($K$9:$K$24,"Sudah Posting")</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="H8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K10" s="7" t="s">
+      <c r="G10" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K11" s="7" t="s">
+      <c r="G11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K12" s="7" t="s">
+      <c r="G12" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K13" s="7" t="s">
+      <c r="G13" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I14" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K14" s="7" t="s">
+      <c r="G14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J15" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K15" s="7" t="s">
+      <c r="G15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J16" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K16" s="7" t="s">
+      <c r="G16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K16" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J17" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K17" s="7" t="s">
+      <c r="G17" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K18" s="7" t="s">
+      <c r="G18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J18" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K18" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I19" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J19" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K19" s="7" t="s">
+      <c r="G19" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J19" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K19" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J20" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K20" s="7" t="s">
+      <c r="G20" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K20" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G21" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J21" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K21" s="7" t="s">
+      <c r="G21" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J22" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K22" s="7" t="s">
+      <c r="G22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="8" t="n">
         <v>26</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I23" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J23" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K23" s="7" t="s">
+      <c r="G23" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J23" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K23" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="E24" s="7" t="s">
+      <c r="D24" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G24" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="K24" s="7" t="s">
+      <c r="G24" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J24" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K24" s="8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1508,86 +1506,82 @@
   <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11"/>
+      <c r="A2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15"/>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+    <row r="13" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11"/>
-    </row>
-    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+    <row r="16" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11"/>
-    </row>
-    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>